<commit_message>
Refactor services to use BaseChatModel and update extractor configurations
- Updated final_markdown_service.py, semantic_router_service.py, and sitemap_extractor_agent_service.py to replace ChatOpenAI with BaseChatModel.
- Removed environment variable checks for API keys and model names, now using get_chat_model for instantiation.
- Updated extractor metadata in automotiveworld_cutoff_audit.json.
- Added new compiled Python files for final_markdown_prompts and semantic_router_prompts.
</commit_message>
<xml_diff>
--- a/output/extracted_urls/automotiveworld/automotiveworld_urls.xlsx
+++ b/output/extracted_urls/automotiveworld/automotiveworld_urls.xlsx
@@ -494,7 +494,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Mostly a product launch with specs and pre-order timing; the body gives only light platform and battery details, not substantive R&amp;D or engineering analysis.</t>
+          <t>Mostly a product launch with specs and marketing features; the body gives only light platform and battery details, not substantive engineering or validation insight.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -535,7 +535,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Body is mainly a brand launch and concept-car reveal with design/theme details, with only brief high-level mention of autonomy and EREVs.</t>
+          <t>Mostly a brand launch and concept reveal; the body gives only high-level mentions of autonomy and EREVs with no real engineering detail.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -567,22 +567,26 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>not_selected</t>
+          <t>selected</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Body is mainly a funding/facility announcement; it mentions battery recycling yields and materials, but gives little engineering detail about the process or validation implications.</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
+          <t>Body gives concrete battery-material recovery and recycling process details with supply-chain and manufacturing implications.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>output/final_markdown/automotiveworld/automotiveworld_final.md</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>skipped_not_selected</t>
+          <t>appended</t>
         </is>
       </c>
     </row>
@@ -608,7 +612,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -617,7 +621,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Body describes an L4 autonomous-driving world model that identifies failure modes, directs targeted data collection, and feeds a training loop with safety and validation implications.</t>
+          <t>The body describes an L4 autonomy development method with self-diagnosis, targeted data collection, and cloud training loop implications for validation and scaling.</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -649,7 +653,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -658,7 +662,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Body is just a forecast teaser with no engineering narrative, mainly subscription prompt and market outlook.</t>
+          <t>Body is just a short forecast blurb with subscription gate, focused on sales/registrations rather than engineering substance.</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -690,7 +694,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -699,7 +703,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Body is just a forecast teaser and subscription gate with no substantive engineering narrative.</t>
+          <t>Body is just a subscription teaser for a production forecast, with no substantive engineering narrative or technical detail.</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
@@ -731,7 +735,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -740,7 +744,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Body is mainly a municipal data-sharing pilot about potholes, with little engineering or validation detail beyond a brief mention of perception systems.</t>
+          <t>It describes a data-sharing pilot for pothole detection, but the body is mostly a city-infrastructure collaboration with little engineering depth.</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
@@ -772,7 +776,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -781,17 +785,13 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Describes ADAS platform integration, safety-certifiable compute consolidation, and centralised vehicle architecture implications.</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>output/final_markdown/automotiveworld/automotiveworld_final.md</t>
-        </is>
-      </c>
+          <t>The body gives concrete ADAS platform and safety-certifiable compute details, including centralized architecture implications and production program timing.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>appended</t>
+          <t>error</t>
         </is>
       </c>
     </row>
@@ -817,7 +817,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -826,7 +826,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Mostly a funding and jobs announcement; the body lacks real battery engineering, validation, or architecture detail.</t>
+          <t>Mostly funding and job-announcement coverage; the body gives little engineering detail beyond a planned battery-cell gigafactory and R&amp;D allocation.</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -867,7 +867,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Mostly a commercial prototype delivery/update with supply-chain and expansion talk; the body lacks substantive engineering or validation detail.</t>
+          <t>Body is mainly a commercial prototype delivery and expansion update, with no substantive engineering, validation, or architecture detail.</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -899,7 +899,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -908,7 +908,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Contains some engineering-relevant circular-economy and battery reuse operations, but the body is mostly business metrics and recycling volumes rather than technical R&amp;D detail.</t>
+          <t>Body is mainly circular-economy and aftersales scale metrics, with little engineering or validation detail beyond battery service and remanufacturing operations.</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
@@ -940,7 +940,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -949,13 +949,17 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Body includes concrete driver-monitoring and unresponsive-driver mitigation tech details with engineering implications for ADAS safety and validation.</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr"/>
+          <t>The body describes an in-vehicle driver monitoring and intervention system update, including camera/sensor detection, unresponsive-driver slowing to stop, and OnStar contact, which has clear engineering and safety relevance.</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>output/final_markdown/automotiveworld/automotiveworld_final.md</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>appended</t>
         </is>
       </c>
     </row>
@@ -981,7 +985,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -990,7 +994,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Body covers SDV cockpit, zonal E/E architecture, ECU reduction, and connectivity/OTA implications with concrete engineering details.</t>
+          <t>The body describes concrete SDV cockpit, zonal E/E, ECU reduction, and RedCap architecture details with engineering implications.</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1026,7 +1030,7 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1035,7 +1039,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>It describes fleet telematics pre-installation logistics, but the body is mostly a partnership/program update with little engineering depth.</t>
+          <t>The body is mainly a fleet telematics pre-installation partnership and logistics note, with little engineering or R&amp;D depth beyond product deployment.</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -1067,7 +1071,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1076,7 +1080,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Mostly a product launch with specs and features; only brief mention of 800V charging and battery monitoring, without deeper engineering substance.</t>
+          <t>Mostly a product launch with range, price, and feature specs; little engineering depth beyond brief architecture mentions.</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
@@ -1108,7 +1112,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1117,7 +1121,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Mostly a launch and manufacturing announcement; the body gives only basic platform/range facts with no substantive engineering or validation detail.</t>
+          <t>Body is mainly a launch announcement with generic EV positioning, not engineering detail beyond platform and range.</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
@@ -1149,7 +1153,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1158,7 +1162,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Mostly a production-site announcement with limited engineering detail beyond high-level ADAS camera localization and R&amp;D center mention.</t>
+          <t>Mostly a manufacturing expansion announcement with localization quotes; the body lacks substantive engineering or validation detail on the camera system itself.</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
@@ -1190,7 +1194,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1199,7 +1203,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>The body is mostly a deployment/partnership announcement with validation timing and fleet scale, but no substantive engineering detail about the autonomous system or test methodology.</t>
+          <t>Body is mostly a program update about AV testing and rollout plans, with little engineering detail beyond validation staffing and fleet scaling.</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
@@ -1231,7 +1235,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1240,7 +1244,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Body is just a brief trade/politics teaser with no engineering or R&amp;D substance.</t>
+          <t>Body is just a short trade-policy teaser with no engineering or R&amp;D substance.</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
@@ -1272,7 +1276,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1281,7 +1285,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Body is a short market/regulatory teaser about large SUVs and pickups, with no substantive engineering or R&amp;D detail.</t>
+          <t>Body is a brief market/regulatory note with no engineering detail beyond import rules and production trends.</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
@@ -1313,7 +1317,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1322,7 +1326,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Mostly a show-and-tell product announcement with specs and event context, not substantive engineering or R&amp;D content.</t>
+          <t>Body is a showroom-style auto show announcement with model/engine specs, not engineering or R&amp;D analysis.</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
@@ -1354,7 +1358,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1363,7 +1367,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Body is about a certified sustainability/carbon-footprint assessment tool for body shops, with little engineering or vehicle R&amp;D substance.</t>
+          <t>Body focuses on sustainability certification and body-shop carbon accounting, not automotive R&amp;D or engineering development.</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
@@ -1395,7 +1399,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1404,7 +1408,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Mostly a market-share update; the body has little engineering detail beyond general MCU and SDV mentions.</t>
+          <t>Body is mainly a market-share ranking and leadership quote, with little engineering or R&amp;D substance beyond brief platform mentions.</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
@@ -1436,7 +1440,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1445,7 +1449,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Body gives concrete software-process maturity evidence for an automotive supplier’s interior lighting development, relevant to SDV engineering and validation readiness.</t>
+          <t>The body has concrete software-process engineering content about Automotive SPICE Level 2, process maturity, and SDV-related development capability.</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1481,7 +1485,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1490,7 +1494,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Body is mainly a live charging demo and deployment promo with performance claims, but no substantive engineering detail beyond headline-level charging specs.</t>
+          <t>Mostly a charging demo/market showcase with little engineering detail beyond headline power figures and no substantive R&amp;D or validation discussion.</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
@@ -1522,7 +1526,7 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1531,7 +1535,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Body contains concrete driveline monitoring, e-drive efficiency, power, axle load/torque and platform-integration details relevant to bus powertrain engineering.</t>
+          <t>The body describes specific driveline monitoring software, e-drive efficiency, and axle/platform integration details relevant to vehicle powertrain engineering and validation.</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1567,7 +1571,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1576,7 +1580,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Mostly a production milestone and plant capability story, with little engineering detail beyond general hybrid transmission manufacturing.</t>
+          <t>Mostly a production milestone and factory promotion; the body gives little engineering detail beyond general lean manufacturing and smart-factory demonstrations.</t>
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
@@ -1608,7 +1612,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1617,7 +1621,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Discusses traction motor magnet supply, recycling, and rare-earth-free motor technology with direct implications for EV powertrain design and supply-chain engineering.</t>
+          <t>Discusses EV traction motor supply-chain engineering, PMSM magnet demand, recycling potential, and rare-earth-free motor technology implications.</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1653,26 +1657,22 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>selected</t>
+          <t>not_selected</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>The body describes a new automotive seating foam material with chemical substitutions, molding, weight/waste reduction, and end-of-life recovery implications.</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>output/final_markdown/automotiveworld/automotiveworld_final.md</t>
-        </is>
-      </c>
+          <t>Body describes a sustainable seating-material production plant and material chemistry, but offers little engineering detail beyond manufacturing and recyclability.</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>appended</t>
+          <t>skipped_not_selected</t>
         </is>
       </c>
     </row>
@@ -1698,7 +1698,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1707,7 +1707,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>A fleet handover story with basic ergonomics and visibility notes, but no substantive engineering, validation, or R&amp;D content.</t>
+          <t>Routine fleet handover with ergonomic and visibility features, but no substantive engineering or R&amp;D content.</t>
         </is>
       </c>
       <c r="H31" t="inlineStr"/>
@@ -1739,7 +1739,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1748,7 +1748,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>A leadership appointment with no substantive engineering, validation, or technical development detail in the body.</t>
+          <t>It is a leadership/design appointment notice with no substantive engineering or R&amp;D detail beyond a general mention of working with engineering teams.</t>
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
@@ -1780,7 +1780,7 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1789,7 +1789,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Mostly a product launch with specs and pricing; little engineering depth beyond basic range, charging, and feature listings.</t>
+          <t>Mostly a launch/spec sheet with pricing, range and features; little engineering depth or R&amp;D insight in the body.</t>
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
@@ -1830,7 +1830,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Body is brand-experience marketing with no engineering, validation, or technical development substance.</t>
+          <t>Body is about brand experience studios and customer engagement, with no engineering or R&amp;D substance.</t>
         </is>
       </c>
       <c r="H34" t="inlineStr"/>
@@ -1862,7 +1862,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -1871,7 +1871,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Body is a leadership/restructuring announcement with no engineering or R&amp;D content.</t>
+          <t>This is mainly a leadership and restructuring announcement with no substantive engineering or R&amp;D content.</t>
         </is>
       </c>
       <c r="H35" t="inlineStr"/>
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>The body discusses large-scale driving data for training, simulation, and validation of an open-source end-to-end autonomy model, with clear engineering and safety implications.</t>
+          <t>The body describes a large-scale driving dataset used to train and validate end-to-end autonomous driving models, with explicit engineering implications for simulation, edge cases, and system safety.</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Body is just a short sales summary with a paywall, offering no engineering or R&amp;D substance.</t>
+          <t>Body is a brief sales summary with no engineering or R&amp;D substance.</t>
         </is>
       </c>
       <c r="H37" t="inlineStr"/>
@@ -1989,7 +1989,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Mostly a brand and product-planning announcement with no real engineering detail beyond naming hybrid/V6 models and a new platform.</t>
+          <t>Mostly a brand/product strategy announcement with model and powertrain plans, but no substantive engineering or validation detail.</t>
         </is>
       </c>
       <c r="H38" t="inlineStr"/>
@@ -2030,7 +2030,7 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -2039,7 +2039,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Mostly a strategy announcement; body lacks engineering depth beyond high-level AI and electrification references.</t>
+          <t>Mostly a strategy/portfolio announcement with sales targets; the body lacks engineering detail beyond high-level AI and electrification mentions.</t>
         </is>
       </c>
       <c r="H39" t="inlineStr"/>
@@ -2071,7 +2071,7 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -2080,7 +2080,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Body includes concrete hybrid architecture, energy management, battery protection and fault-prediction details relevant to powertrain and systems engineering.</t>
+          <t>Body includes concrete hybrid architecture, AI energy management, efficiency metrics, and fault prediction details relevant to vehicle systems engineering.</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2116,7 +2116,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -2125,7 +2125,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Body gives concrete solid-state battery patent activity, filings, grants, and technical focus areas like electrodes, electrolytes, safety, and thermal regulation.</t>
+          <t>Body contains substantive solid-state battery patent activity and electrode/electrolyte R&amp;D trends relevant to battery engineering.</t>
         </is>
       </c>
       <c r="H41" t="inlineStr"/>
@@ -2157,7 +2157,7 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -2166,7 +2166,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Mostly a facility announcement with only brief product specs; little engineering depth beyond assembly and supply-chain context.</t>
+          <t>Mentions charging hardware and testing, but the body is mostly a plant-opening announcement with little engineering detail.</t>
         </is>
       </c>
       <c r="H42" t="inlineStr"/>
@@ -2198,7 +2198,7 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -2207,7 +2207,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>The body contains concrete engineering details on e-axle integration, dual-motor drivetrains, gearbox design, MCS charging, payload, and power take-off implications.</t>
+          <t>The body contains concrete engineering details on e-axle integration, battery packaging, charging power, drivetrain architecture, and PTO use, which are useful for automotive R&amp;D.</t>
         </is>
       </c>
       <c r="H43" t="inlineStr"/>
@@ -2239,7 +2239,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Body describes automated V2G/TLS security validation for EV charging communication, with CI/CD workflow and standards implications for development.</t>
+          <t>The body describes automated V2G/TLS security testing for charging communication, with validation workflow and standards details that are directly useful to EV engineering teams.</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2284,7 +2284,7 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -2293,7 +2293,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>The body is mainly about charging-network payments and uptime, with no substantive vehicle engineering, validation, or platform R&amp;D content.</t>
+          <t>Body is mainly about charging-network payments and uptime targets, with no substantive automotive engineering or R&amp;D detail.</t>
         </is>
       </c>
       <c r="H45" t="inlineStr"/>
@@ -2325,7 +2325,7 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -2334,7 +2334,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Mostly a facility consolidation and operations announcement; the body has little engineering detail beyond generic manufacturing/R&amp;D space.</t>
+          <t>The body is mainly a facility consolidation and logistics announcement, with only generic mentions of R&amp;D and manufacturing and no real engineering detail.</t>
         </is>
       </c>
       <c r="H46" t="inlineStr"/>
@@ -2366,7 +2366,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -2375,17 +2375,13 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Body includes concrete engineering changes—800V architecture, battery chemistry, steer-by-wire, drive units, and OTA V2G/V2H—relevant to vehicle platform development.</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>output/final_markdown/automotiveworld/automotiveworld_final.md</t>
-        </is>
-      </c>
+          <t>The body includes real engineering substance on 800V architecture, battery chemistry, charging, recuperation, steer-by-wire, and MB.OS integration.</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr">
         <is>
-          <t>appended</t>
+          <t>error</t>
         </is>
       </c>
     </row>
@@ -2411,7 +2407,7 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -2420,7 +2416,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Body is about logistics software and supply-chain planning, with no substantive vehicle engineering, validation, or R&amp;D detail.</t>
+          <t>The body is about logistics network planning software and carbon-efficiency operations, not automotive R&amp;D or engineering design/validation.</t>
         </is>
       </c>
       <c r="H48" t="inlineStr"/>
@@ -2461,17 +2457,13 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>The body gives concrete engineering changes to 800V architecture, charging hardware, thermal/cabling impacts, and battery charge-control software.</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>output/final_markdown/automotiveworld/automotiveworld_final.md</t>
-        </is>
-      </c>
+          <t>Contains concrete engineering changes to 800V architecture, charging hardware, thermal/cabling impacts, and adaptive battery software affecting validation and battery health.</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
-          <t>appended</t>
+          <t>error</t>
         </is>
       </c>
     </row>
@@ -2506,7 +2498,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Body is just a production forecast teaser with no engineering or R&amp;D detail beyond volume data.</t>
+          <t>Body is just a production-data teaser with no engineering or R&amp;D substance.</t>
         </is>
       </c>
       <c r="H50" t="inlineStr"/>
@@ -2538,7 +2530,7 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -2547,7 +2539,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Body is mainly a CEO appointment and scaling/profitability news, with little engineering or technical detail.</t>
+          <t>Mostly an executive appointment and profitability/scaling news, with no substantive engineering or R&amp;D detail in the body.</t>
         </is>
       </c>
       <c r="H51" t="inlineStr"/>
@@ -2579,7 +2571,7 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -2588,7 +2580,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Mostly an investment and deployment announcement; the body gives only high-level platform claims with no real engineering detail.</t>
+          <t>Mostly investment and fleet-deployment news with only high-level platform claims; no substantive engineering or validation detail in the body.</t>
         </is>
       </c>
       <c r="H52" t="inlineStr"/>
@@ -2629,7 +2621,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Body is mainly a responsible sourcing policy and supplier compliance update, not automotive engineering or R&amp;D substance.</t>
+          <t>Body is mainly a responsible sourcing policy and supplier compliance note, with little engineering or R&amp;D substance.</t>
         </is>
       </c>
       <c r="H53" t="inlineStr"/>
@@ -2661,7 +2653,7 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -2670,7 +2662,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Mostly an attached data/forecast teaser with only brief methodology and no substantive engineering or R&amp;D narrative.</t>
+          <t>Mostly an attached forecast/data teaser with no substantive engineering narrative; the body is just methodology and section headers.</t>
         </is>
       </c>
       <c r="H54" t="inlineStr"/>
@@ -2702,7 +2694,7 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -2711,7 +2703,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Mostly a launch/spec overview with pricing, range, and features; the body lacks deeper engineering or validation substance.</t>
+          <t>Mostly a launch/spec announcement with range, charging and feature list, with little engineering depth beyond basic platform and ADAS mentions.</t>
         </is>
       </c>
       <c r="H55" t="inlineStr"/>
@@ -2752,7 +2744,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Mostly a vehicle announcement with performance specs and trim details, not engineering or R&amp;D analysis.</t>
+          <t>Mostly a product announcement with specs and styling; the body has little engineering or validation substance beyond basic component and performance details.</t>
         </is>
       </c>
       <c r="H56" t="inlineStr"/>
@@ -2793,7 +2785,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Body gives concrete coating material, durability, optical, and process details relevant to display engineering and PFAS compliance.</t>
+          <t>Body gives concrete materials and validation details for display coatings, including PFAS-free formulation, abrasion/UV durability, hardness, and application processes relevant to automotive engineering.</t>
         </is>
       </c>
       <c r="H57" t="inlineStr"/>
@@ -2825,22 +2817,26 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>not_selected</t>
+          <t>selected</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Body is mainly a hub opening announcement with general software and connected-services work, but little concrete engineering or validation detail.</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr"/>
+          <t>The body describes software, cloud, and cybersecurity development for connected vehicle apps and services, which is directly relevant to automotive engineering work.</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>output/final_markdown/automotiveworld/automotiveworld_final.md</t>
+        </is>
+      </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>skipped_not_selected</t>
+          <t>appended</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2862,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
@@ -2875,7 +2871,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Body is mainly labour-rights and political reporting about factory conditions, with no meaningful automotive engineering or R&amp;D substance.</t>
+          <t>Body is about labor-rights allegations and politics at a factory site, with no substantive automotive engineering or R&amp;D content.</t>
         </is>
       </c>
       <c r="H59" t="inlineStr"/>
@@ -2907,7 +2903,7 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
@@ -2916,13 +2912,17 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>The body discusses engineering headcount cuts, faster 24-month vehicle development cycles, and China-linked cost/architecture pressures affecting Renault’s product development.</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr"/>
+          <t>Body discusses engineering workforce cuts tied to faster vehicle development, platform strategy, and China cost/speed competition, which has clear R&amp;D and engineering implications.</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>output/final_markdown/automotiveworld/automotiveworld_final.md</t>
+        </is>
+      </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>appended</t>
         </is>
       </c>
     </row>
@@ -2948,26 +2948,22 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>selected</t>
+          <t>not_selected</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>The body includes concrete engineering choices—600-part vehicle architecture, paintless composite panels, battery variants, and an unconventional manufacturing approach that affects production and service.</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>output/final_markdown/automotiveworld/automotiveworld_final.md</t>
-        </is>
-      </c>
+          <t>Includes some engineering/production details like component count, battery sizes, and paintless composite body manufacturing, but the body is mostly a startup funding and launch/pricing story.</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr">
         <is>
-          <t>appended</t>
+          <t>skipped_not_selected</t>
         </is>
       </c>
     </row>
@@ -3002,7 +2998,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Body is mainly a legal/reputation dispute and market competition story, with no substantive engineering, R&amp;D, or vehicle development content.</t>
+          <t>Body is mainly about legal/PR conflict and market competition, with no substantive engineering, validation, or vehicle development content.</t>
         </is>
       </c>
       <c r="H62" t="inlineStr"/>
@@ -3075,7 +3071,7 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -3084,7 +3080,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Body is just a brief lineup-reduction note with no engineering detail beyond a subscription prompt.</t>
+          <t>Body is a brief business note about lineup reduction with no engineering or R&amp;D substance beyond reallocating investment.</t>
         </is>
       </c>
       <c r="H64" t="inlineStr"/>
@@ -3125,7 +3121,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Body is just attached datasets, section headings, and a subscription gate, with no substantive engineering or R&amp;D narrative.</t>
+          <t>Body is mostly attached datasets, section headings, and a subscribe prompt, with no substantive engineering narrative.</t>
         </is>
       </c>
       <c r="H65" t="inlineStr"/>
@@ -3157,7 +3153,7 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
@@ -3166,7 +3162,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Discusses second-life battery packs for plant energy storage, but the body is mostly a partnership announcement with limited engineering detail.</t>
+          <t>Body is mainly a business tie-up about second-life batteries for plant energy storage, with little engineering or validation detail.</t>
         </is>
       </c>
       <c r="H66" t="inlineStr"/>
@@ -3198,7 +3194,7 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
@@ -3207,7 +3203,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Mostly a funding and deployment announcement; the body gives only high-level autonomous transit claims with no real engineering detail.</t>
+          <t>Mostly a funding and rollout announcement; the body gives only high-level AV network claims and no substantive engineering or validation detail.</t>
         </is>
       </c>
       <c r="H67" t="inlineStr"/>
@@ -3239,7 +3235,7 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
@@ -3248,7 +3244,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Mostly financial and restructuring news with only brief, high-level mentions of product units and EV ramp-up, not engineering detail.</t>
+          <t>Mostly a financial turnaround and restructuring report, with only brief mention of EV ramp-up and business-unit sales but no substantive engineering or R&amp;D detail.</t>
         </is>
       </c>
       <c r="H68" t="inlineStr"/>
@@ -3289,7 +3285,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Mostly sales rollout and award updates; the body only gives a few vehicle specs and a battery safety claim without engineering depth.</t>
+          <t>Body is mainly rollout, deliveries, awards, and launch plans; only a brief battery/charging mention with no engineering depth.</t>
         </is>
       </c>
       <c r="H69" t="inlineStr"/>
@@ -3321,7 +3317,7 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>34</v>
+        <v>56</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
@@ -3330,7 +3326,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Mostly a preliminary business framework; the body gives only high-level automation intentions with no real engineering detail or validation implications.</t>
+          <t>The body mentions semi-autonomous navigation and vehicle-platform upgrades, but it’s only a preliminary cooperation framework with no engineering detail or validation substance.</t>
         </is>
       </c>
       <c r="H70" t="inlineStr"/>
@@ -3362,22 +3358,26 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>55</v>
+        <v>74</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>not_selected</t>
+          <t>selected</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Contains some deployment detail on private cellular coverage for autonomous logistics, but it is mainly a site connectivity install with little automotive engineering depth.</t>
-        </is>
-      </c>
-      <c r="H71" t="inlineStr"/>
+          <t>Body includes concrete networking and RF deployment details for autonomous vehicle operations in an industrial setting, with engineering relevance to connectivity and coverage challenges.</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>output/final_markdown/automotiveworld/automotiveworld_final.md</t>
+        </is>
+      </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>skipped_not_selected</t>
+          <t>appended</t>
         </is>
       </c>
     </row>
@@ -3403,7 +3403,7 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
@@ -3412,7 +3412,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>The body discusses automotive chiplet architecture, packaging, testing, and standards for ADAS and software-defined vehicles, which is directly useful engineering content.</t>
+          <t>The body gives concrete engineering context on automotive chiplet packaging, interconnection, testing, and automotive-grade standards for ADAS/software-defined vehicles.</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -3448,7 +3448,7 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
@@ -3457,13 +3457,17 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>The body discusses semiconductor fabrication, chip process nodes, tape-out delays, and supply-chain constraints that directly affect vehicle compute and platform engineering.</t>
-        </is>
-      </c>
-      <c r="H73" t="inlineStr"/>
+          <t>Body contains substantive semiconductor and vehicle compute details, including 2nm fab plans, AI5/AI6 chip delays, and manufacturing constraints that affect automotive engineering.</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>output/final_markdown/automotiveworld/automotiveworld_final.md</t>
+        </is>
+      </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>appended</t>
         </is>
       </c>
     </row>
@@ -3489,26 +3493,22 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>selected</t>
+          <t>not_selected</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>The body discusses semiconductor fab equipment procurement, process capability, and supply-chain implications for custom AI chips, which is relevant to automotive engineering and platform teams.</t>
-        </is>
-      </c>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>output/final_markdown/automotiveworld/automotiveworld_final.md</t>
-        </is>
-      </c>
+          <t>Body is mainly a procurement/status update on an AI chip fab, with little concrete engineering detail beyond supplier outreach and timelines.</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr"/>
       <c r="I74" t="inlineStr">
         <is>
-          <t>appended</t>
+          <t>skipped_not_selected</t>
         </is>
       </c>
     </row>
@@ -3534,7 +3534,7 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
@@ -3543,7 +3543,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Mentions electric truck range and charging infrastructure, but the body is mostly a tour/demo announcement with limited engineering detail.</t>
+          <t>Mostly a tour/market-readiness promo with little engineering detail beyond basic truck specs and charging claims.</t>
         </is>
       </c>
       <c r="H75" t="inlineStr"/>
@@ -3584,17 +3584,13 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Body describes an ADAS sensor-based road-defect detection system using cameras/LiDAR, accuracy results, and deployment implications for safety and validation.</t>
-        </is>
-      </c>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>output/final_markdown/automotiveworld/automotiveworld_final.md</t>
-        </is>
-      </c>
+          <t>The body explains an ADAS-sensor-based roadway defect detection system with pilot scale, sensor types, accuracy, and workflow implications.</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr"/>
       <c r="I76" t="inlineStr">
         <is>
-          <t>appended</t>
+          <t>error</t>
         </is>
       </c>
     </row>
@@ -3620,7 +3616,7 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
@@ -3629,7 +3625,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Mostly a sales milestone and strategy statement, with only a brief note about a battery update and range change.</t>
+          <t>Mostly sales and strategy reporting with only a brief mention of a battery update, lacking substantive engineering detail.</t>
         </is>
       </c>
       <c r="H77" t="inlineStr"/>
@@ -3661,26 +3657,22 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>selected</t>
+          <t>not_selected</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>The body describes an automotive motor-control chip architecture, sensorless FOC at zero speed, and ECU miniaturization implications for pumps and fans.</t>
-        </is>
-      </c>
-      <c r="H78" t="inlineStr">
-        <is>
-          <t>output/final_markdown/automotiveworld/automotiveworld_final.md</t>
-        </is>
-      </c>
+          <t>Useful powertrain/control integration details, but the article is mainly a product announcement with limited engineering depth beyond MCU-plus-driver integration and sensorless motor control.</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr"/>
       <c r="I78" t="inlineStr">
         <is>
-          <t>appended</t>
+          <t>skipped_not_selected</t>
         </is>
       </c>
     </row>
@@ -3706,7 +3698,7 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -3715,17 +3707,13 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Body discusses an SRS ECU calibration fault, unintended airbag deployment triggers, and dealer reprogramming—clear validation/safety engineering relevance.</t>
-        </is>
-      </c>
-      <c r="H79" t="inlineStr">
-        <is>
-          <t>output/final_markdown/automotiveworld/automotiveworld_final.md</t>
-        </is>
-      </c>
+          <t>Body describes an SRS ECU calibration defect, unintended airbag deployment risk, injury reports, and the software fix path, which is directly relevant to vehicle safety engineering and validation.</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr"/>
       <c r="I79" t="inlineStr">
         <is>
-          <t>appended</t>
+          <t>error</t>
         </is>
       </c>
     </row>
@@ -3760,7 +3748,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>The body contains concrete engineering content on Ford’s zonal architecture, in-house software controls, ADAS integration, and castings for the UEV platform.</t>
+          <t>Body includes concrete engineering content on Ford’s zonal architecture, in-house software controls, ADAS, large castings, and platform industrialization.</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -3796,26 +3784,22 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>74</v>
+        <v>46</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>selected</t>
+          <t>not_selected</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>The body discusses joint fuel-cell truck development, platform integration, and cost/manufacturing optimization, which are meaningful engineering topics for vehicle R&amp;D.</t>
-        </is>
-      </c>
-      <c r="H81" t="inlineStr">
-        <is>
-          <t>output/final_markdown/automotiveworld/automotiveworld_final.md</t>
-        </is>
-      </c>
+          <t>A real vehicle engineering project is described, but the body stays high-level on hydrogen use and cost reduction with no detailed R&amp;D, validation, or architecture substance.</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr">
         <is>
-          <t>appended</t>
+          <t>skipped_not_selected</t>
         </is>
       </c>
     </row>
@@ -3841,7 +3825,7 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
@@ -3850,7 +3834,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Mostly a product reveal with specs and feature lists; little engineering depth beyond range, charging, and infotainment updates.</t>
+          <t>Mostly a vehicle update with range, trims, and feature specs; the body lacks substantive engineering or validation detail.</t>
         </is>
       </c>
       <c r="H82" t="inlineStr"/>
@@ -3891,7 +3875,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>The body is mainly about carbon-footprint reduction and sourcing, with little engineering detail beyond materials and renewable energy use.</t>
+          <t>Body is mainly carbon-footprint and sourcing claims, with no real battery engineering, validation, or vehicle-system technical detail.</t>
         </is>
       </c>
       <c r="H83" t="inlineStr"/>
@@ -3923,7 +3907,7 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
@@ -3932,7 +3916,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Body is mainly an aftersales/service-package announcement with no substantive engineering or R&amp;D detail.</t>
+          <t>Mostly an aftersales/service packaging update with little engineering or validation detail beyond general maintenance coverage.</t>
         </is>
       </c>
       <c r="H84" t="inlineStr"/>
@@ -3964,7 +3948,7 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
@@ -3973,7 +3957,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Body is just a subscription teaser and section list, with no substantive engineering narrative.</t>
+          <t>The body is just an outline plus a subscription gate, with no substantive engineering or R&amp;D content.</t>
         </is>
       </c>
       <c r="H85" t="inlineStr"/>
@@ -4005,7 +3989,7 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="F86" t="inlineStr">
         <is>
@@ -4014,17 +3998,13 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Discusses Ford’s universal EV platform, advanced electrical architecture, and industrialization/cost challenges that directly affect engineering and platform development.</t>
-        </is>
-      </c>
-      <c r="H86" t="inlineStr">
-        <is>
-          <t>output/final_markdown/automotiveworld/automotiveworld_final.md</t>
-        </is>
-      </c>
+          <t>The body contains substantive EV platform and electrical-architecture discussion, including technical execution, cost structure, and industrialisation implications for Ford’s development program.</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr"/>
       <c r="I86" t="inlineStr">
         <is>
-          <t>appended</t>
+          <t>error</t>
         </is>
       </c>
     </row>
@@ -4050,7 +4030,7 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F87" t="inlineStr">
         <is>
@@ -4059,7 +4039,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Body is just a short trade/tariff note with no engineering or R&amp;D substance.</t>
+          <t>Body is just a brief trade-policy blurb with no engineering or R&amp;D substance.</t>
         </is>
       </c>
       <c r="H87" t="inlineStr"/>
@@ -4091,22 +4071,26 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>not_selected</t>
+          <t>selected</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Contains some ADAS and crash-safety engineering details, but it is mainly a vehicle safety-rating announcement rather than a deep R&amp;D or validation article.</t>
-        </is>
-      </c>
-      <c r="H88" t="inlineStr"/>
+          <t>Contains concrete ADAS and lighting engineering changes tied to crash-test and detection performance, not just a launch announcement.</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>output/final_markdown/automotiveworld/automotiveworld_final.md</t>
+        </is>
+      </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>skipped_not_selected</t>
+          <t>appended</t>
         </is>
       </c>
     </row>
@@ -4132,7 +4116,7 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
@@ -4141,7 +4125,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Mostly a site transformation and workforce news item, with only brief mention of R&amp;D prototypes and no substantive engineering detail.</t>
+          <t>The body mainly describes a plant restructuring and jobs plan, with only a small mention of a 3D printing R&amp;D prototype center and little engineering detail.</t>
         </is>
       </c>
       <c r="H89" t="inlineStr"/>
@@ -4173,7 +4157,7 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
@@ -4182,7 +4166,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Contains concrete ADAS architecture, Qualcomm mass-production deployment, and simulation/validation details relevant to engineering teams.</t>
+          <t>The body contains concrete ADAS architecture and validation details, including end-to-end deployment, Qualcomm/Nvidia platform support, semantic perception, and simulation-based scenario testing.</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -4227,7 +4211,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Mostly a tyre fitment announcement with limited engineering detail and no broader R&amp;D or architecture implications.</t>
+          <t>Mostly an OE tyre fitment announcement with generic performance claims and little substantive engineering detail beyond basic tread, noise, and rolling-resistance notes.</t>
         </is>
       </c>
       <c r="H91" t="inlineStr"/>
@@ -4259,7 +4243,7 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -4268,7 +4252,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Mentions pedal-by-wire, swappable batteries, regenerative braking, OTA updates and diagnostics, but the body is mainly a commercial micromobility launch with limited engineering depth.</t>
+          <t>Contains some engineering details like pedal-by-wire, swappable batteries, regen braking and OTA diagnostics, but the article is mainly a commercial launch/partnership announcement with limited R&amp;D depth.</t>
         </is>
       </c>
       <c r="H92" t="inlineStr"/>
@@ -4300,26 +4284,22 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>selected</t>
+          <t>not_selected</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>The body includes engineering-relevant AI use cases like validation, predictive maintenance, cyber defense for connected vehicles, and cloud infrastructure affecting development and resilience.</t>
-        </is>
-      </c>
-      <c r="H93" t="inlineStr">
-        <is>
-          <t>output/final_markdown/automotiveworld/automotiveworld_final.md</t>
-        </is>
-      </c>
+          <t>Mentions AI validation and connected-vehicle cyber defence, but the body is mostly a high-level partnership and infrastructure rollout with little engineering depth.</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr"/>
       <c r="I93" t="inlineStr">
         <is>
-          <t>appended</t>
+          <t>skipped_not_selected</t>
         </is>
       </c>
     </row>
@@ -4354,7 +4334,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Body is mostly about defence policy and OEM business strategy, with only broad mentions of manufacturing capacity and tolerances, not automotive R&amp;D or engineering detail.</t>
+          <t>Body is mainly about OEM business/policy and defence capacity talks, with no substantive automotive engineering or R&amp;D detail.</t>
         </is>
       </c>
       <c r="H94" t="inlineStr"/>
@@ -4386,7 +4366,7 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
@@ -4395,7 +4375,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Mostly policy and trade-access lobbying; the body lacks technical engineering detail or R&amp;D substance.</t>
+          <t>Body is mainly trade and industrial policy lobbying, with little engineering or R&amp;D substance beyond broad EV/manufacturing implications.</t>
         </is>
       </c>
       <c r="H95" t="inlineStr"/>
@@ -4436,7 +4416,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>A product launch with pricing and range/payload details, but no substantive engineering, validation, or architecture discussion in the body.</t>
+          <t>A product launch with payload, range, and pricing details; the body lacks substantive engineering or validation discussion.</t>
         </is>
       </c>
       <c r="H96" t="inlineStr"/>
@@ -4468,7 +4448,7 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
@@ -4477,7 +4457,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Body is mainly a consumer in-car services partnership announcement with no substantive engineering, validation, or architecture detail.</t>
+          <t>Mostly a connected-services partnership announcement with no substantive engineering or validation detail.</t>
         </is>
       </c>
       <c r="H97" t="inlineStr"/>
@@ -4509,7 +4489,7 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
@@ -4518,7 +4498,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Mostly an order/pricing and launch announcement; the body gives specs but little engineering depth or R&amp;D insight.</t>
+          <t>Mostly a launch/spec announcement with pricing and range details; little engineering analysis or R&amp;D substance in the body.</t>
         </is>
       </c>
       <c r="H98" t="inlineStr"/>
@@ -4559,7 +4539,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Mostly a rental-car checkout and payment workflow announcement; the body has little engineering depth beyond infotainment integration.</t>
+          <t>Body describes a rental checkout and add-on upsell tool in infotainment, with little engineering or automotive R&amp;D substance.</t>
         </is>
       </c>
       <c r="H99" t="inlineStr"/>
@@ -4591,7 +4571,7 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
@@ -4600,7 +4580,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Body outlines a technical distributed architecture for managing connected-vehicle data at scale, with edge/cloud/peer-to-peer layers and engineering impacts on energy and network load.</t>
+          <t>The body lays out a concrete distributed vehicle-data architecture with peer-to-peer, edge, and cloud layers plus scalability and energy-efficiency implications.</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -4636,7 +4616,7 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
@@ -4645,7 +4625,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Policy commentary on EU transport energy shares and biofuel caps, with no substantive automotive engineering or R&amp;D content.</t>
+          <t>Policy and energy-mix commentary with no substantive automotive engineering, validation, or system-design content.</t>
         </is>
       </c>
       <c r="H101" t="inlineStr"/>
@@ -4677,7 +4657,7 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
@@ -4686,7 +4666,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>This is an editorial calendar/listing page with schedules and link lists, not substantive engineering content.</t>
+          <t>This is an editorial schedule/index page with link listings and dates, not substantive engineering content.</t>
         </is>
       </c>
       <c r="H102" t="inlineStr"/>
@@ -4759,7 +4739,7 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F104" t="inlineStr">
         <is>
@@ -4768,7 +4748,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Paywall/login prompt with no article narrative or engineering content in the body.</t>
+          <t>Paywalled login/subscribe page with no article narrative or engineering content.</t>
         </is>
       </c>
       <c r="H104" t="inlineStr"/>
@@ -4809,7 +4789,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Paywalled login prompt with no article body or engineering content.</t>
+          <t>No article content is present; this is only a subscription/login prompt.</t>
         </is>
       </c>
       <c r="H105" t="inlineStr"/>
@@ -4841,7 +4821,7 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
@@ -4850,7 +4830,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>No article content is present; it is just a subscription/login gate.</t>
+          <t>No article content; just a subscription/login prompt with no engineering narrative.</t>
         </is>
       </c>
       <c r="H106" t="inlineStr"/>
@@ -5243,7 +5223,7 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
@@ -5252,7 +5232,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>Body is just a dated outlook index with no substantive engineering article or technical narrative.</t>
+          <t>Body is just a date list for an OEM outlook page, with no engineering narrative or technical content.</t>
         </is>
       </c>
       <c r="H116" t="inlineStr"/>
@@ -5334,7 +5314,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>Body is just a date list for a production data index page, with no article narrative or engineering substance.</t>
+          <t>This is just a production data index with dates and no substantive article or engineering narrative.</t>
         </is>
       </c>
       <c r="H118" t="inlineStr"/>
@@ -5448,7 +5428,7 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F121" t="inlineStr">
         <is>
@@ -5457,7 +5437,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>This is just an archive/date list with no article narrative or engineering content.</t>
+          <t>This is just a date-based archive/listing page with no substantive article narrative or engineering content.</t>
         </is>
       </c>
       <c r="H121" t="inlineStr"/>
@@ -5498,7 +5478,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>This is just a research archive/index page with dates and navigation, not substantive engineering content.</t>
+          <t>This is just a research archive listing dates and navigation, with no substantive article narrative or engineering content.</t>
         </is>
       </c>
       <c r="H122" t="inlineStr"/>

</xml_diff>